<commit_message>
Add WhatsApp Web AI Bot, 5 Wholesale Categories, NEXT Pagination, Mobile Admin #add/#delete Commands, and Executive Stock Reports
</commit_message>
<xml_diff>
--- a/garment_catalog.xlsx
+++ b/garment_catalog.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -651,6 +650,156 @@
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>girls_sharara_purple_783.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kids Dresses</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Smocked Puff Sleeve Satin Party Gown</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>690</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>24, 26, 28, 30, 32, 34</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Elegant girls satin party gown featuring a smocked elasticated bodice, puff sleeves, flower corsage details on shoulder and waist belt. Colors: Deep Purple, Royal Blue, Hot Pink.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>kids_smocked_puff_sleeve_gown.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kids Dresses</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Red Rose Garland Off-Shoulder Satin Frock</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>680</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>22, 24, 26, 28, 30, 32</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Charming girls satin party frock decorated with a striking horizontal red rose bouquet across the chest and a pleated flared skirt. Colors: Off-White, Lavender, Pastel Yellow, Cream Gold.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>kids_red_rose_garland_satin_frock.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kids Dresses</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cream Rose Corsage Off-Shoulder Satin Frock</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>690</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>24, 26, 28, 30, 32, 34</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Gorgeous girls off-shoulder satin flared frock with prominent cream-yellow rose corsage bouquet across the neck. Colors: Navy Blue, Bright Pink, Deep Magenta.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>kids_yellow_rose_garland_satin_frock.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kids Dresses</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Shimmer Satin Floral Neckline Ball Gown</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>720</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>24, 26, 28, 30, 32, 34</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Premium shimmering satin floor-length ball gown featuring an intricate 3D floral appliqued neckline and matching waist bow. Colors: Mint Green, Pastel Pink, Shimmer Lavender.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>kids_shimmer_floral_neck_ball_gown.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Kids Dresses</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pleated Satin Gown with Flower Sleeves &amp; Bow</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>710</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>24, 26, 28, 30, 32, 34</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Stylish girls box-pleated satin gown featuring 3D floral sleeve embellishments and a center waist bow accent. Colors: Crimson Red, Emerald Green, Warm Bronze.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>kids_pleated_shoulder_flower_satin_gown.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>